<commit_message>
fix: drop admin-only internal column from TID upload sample
</commit_message>
<xml_diff>
--- a/src/main/resources/sample/tids_sample.xlsx
+++ b/src/main/resources/sample/tids_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,11 +477,6 @@
           <t>processor</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>internal</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -540,11 +535,6 @@
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>